<commit_message>
att detalhes produtos COM SQL CERTO2
</commit_message>
<xml_diff>
--- a/public/deltahes_item_ativos.xlsx
+++ b/public/deltahes_item_ativos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luis.h\Desktop\pedido-de-venda-producao\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DBDA6D4-8614-4CF4-BC15-F2666C0464FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419FDD45-8C19-471F-BE17-288A31318890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="585" yWindow="945" windowWidth="15375" windowHeight="7875" xr2:uid="{C5CD4D3D-D302-43D7-A321-16F939601549}"/>
   </bookViews>
@@ -827,19 +827,19 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
         <v>122</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
       </c>
       <c r="K1" t="s">
         <v>9</v>
@@ -907,19 +907,19 @@
         <v>24</v>
       </c>
       <c r="F2">
+        <v>2530</v>
+      </c>
+      <c r="G2">
+        <v>27</v>
+      </c>
+      <c r="H2">
+        <v>21</v>
+      </c>
+      <c r="I2">
+        <v>11</v>
+      </c>
+      <c r="J2">
         <v>36</v>
-      </c>
-      <c r="G2">
-        <v>2530</v>
-      </c>
-      <c r="H2">
-        <v>27</v>
-      </c>
-      <c r="I2">
-        <v>21</v>
-      </c>
-      <c r="J2">
-        <v>11</v>
       </c>
       <c r="K2">
         <v>17898681350015</v>
@@ -977,20 +977,20 @@
       <c r="E3">
         <v>24</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3">
+        <v>2530</v>
+      </c>
+      <c r="G3">
+        <v>27</v>
+      </c>
+      <c r="H3">
+        <v>21</v>
+      </c>
+      <c r="I3">
+        <v>11</v>
+      </c>
+      <c r="J3" t="s">
         <v>123</v>
-      </c>
-      <c r="G3">
-        <v>2530</v>
-      </c>
-      <c r="H3">
-        <v>27</v>
-      </c>
-      <c r="I3">
-        <v>21</v>
-      </c>
-      <c r="J3">
-        <v>11</v>
       </c>
       <c r="K3">
         <v>17898681350015</v>
@@ -1049,19 +1049,19 @@
         <v>96</v>
       </c>
       <c r="F4">
+        <v>2750</v>
+      </c>
+      <c r="G4">
+        <v>25.3</v>
+      </c>
+      <c r="H4">
+        <v>20</v>
+      </c>
+      <c r="I4">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="J4">
         <v>36</v>
-      </c>
-      <c r="G4">
-        <v>2750</v>
-      </c>
-      <c r="H4">
-        <v>25.3</v>
-      </c>
-      <c r="I4">
-        <v>20</v>
-      </c>
-      <c r="J4">
-        <v>17.600000000000001</v>
       </c>
       <c r="K4">
         <v>17898681350039</v>
@@ -1120,19 +1120,19 @@
         <v>24</v>
       </c>
       <c r="F5">
+        <v>1570</v>
+      </c>
+      <c r="G5">
+        <v>28.3</v>
+      </c>
+      <c r="H5">
+        <v>20</v>
+      </c>
+      <c r="I5">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="J5">
         <v>36</v>
-      </c>
-      <c r="G5">
-        <v>1570</v>
-      </c>
-      <c r="H5">
-        <v>28.3</v>
-      </c>
-      <c r="I5">
-        <v>20</v>
-      </c>
-      <c r="J5">
-        <v>17.600000000000001</v>
       </c>
       <c r="K5">
         <v>17898681350060</v>
@@ -1190,20 +1190,20 @@
       <c r="E6">
         <v>24</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6">
+        <v>1570</v>
+      </c>
+      <c r="G6">
+        <v>28.3</v>
+      </c>
+      <c r="H6">
+        <v>20</v>
+      </c>
+      <c r="I6">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="J6" t="s">
         <v>123</v>
-      </c>
-      <c r="G6">
-        <v>1570</v>
-      </c>
-      <c r="H6">
-        <v>28.3</v>
-      </c>
-      <c r="I6">
-        <v>20</v>
-      </c>
-      <c r="J6">
-        <v>17.600000000000001</v>
       </c>
       <c r="K6">
         <v>17898681350060</v>
@@ -1262,19 +1262,19 @@
         <v>48</v>
       </c>
       <c r="F7">
+        <v>4800</v>
+      </c>
+      <c r="G7">
+        <v>38.5</v>
+      </c>
+      <c r="H7">
+        <v>19.5</v>
+      </c>
+      <c r="I7">
+        <v>21.7</v>
+      </c>
+      <c r="J7">
         <v>36</v>
-      </c>
-      <c r="G7">
-        <v>4800</v>
-      </c>
-      <c r="H7">
-        <v>38.5</v>
-      </c>
-      <c r="I7">
-        <v>19.5</v>
-      </c>
-      <c r="J7">
-        <v>21.7</v>
       </c>
       <c r="K7">
         <v>17898681350084</v>
@@ -1332,20 +1332,20 @@
       <c r="E8">
         <v>48</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8">
+        <v>4800</v>
+      </c>
+      <c r="G8">
+        <v>38.5</v>
+      </c>
+      <c r="H8">
+        <v>19.5</v>
+      </c>
+      <c r="I8">
+        <v>21.7</v>
+      </c>
+      <c r="J8" t="s">
         <v>123</v>
-      </c>
-      <c r="G8">
-        <v>4800</v>
-      </c>
-      <c r="H8">
-        <v>38.5</v>
-      </c>
-      <c r="I8">
-        <v>19.5</v>
-      </c>
-      <c r="J8">
-        <v>21.7</v>
       </c>
       <c r="K8">
         <v>17898681350084</v>
@@ -1403,20 +1403,20 @@
       <c r="E9">
         <v>36</v>
       </c>
-      <c r="F9" t="s">
-        <v>123</v>
+      <c r="F9">
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>0.38</v>
       </c>
       <c r="H9">
-        <v>0.38</v>
+        <v>0.19</v>
       </c>
       <c r="I9">
         <v>0.19</v>
       </c>
-      <c r="J9">
-        <v>0.19</v>
+      <c r="J9" t="s">
+        <v>123</v>
       </c>
       <c r="K9">
         <v>17898681350121</v>
@@ -1475,19 +1475,19 @@
         <v>24</v>
       </c>
       <c r="F10">
+        <v>2330</v>
+      </c>
+      <c r="G10">
+        <v>22</v>
+      </c>
+      <c r="H10">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="I10">
+        <v>21.7</v>
+      </c>
+      <c r="J10">
         <v>36</v>
-      </c>
-      <c r="G10">
-        <v>2330</v>
-      </c>
-      <c r="H10">
-        <v>22</v>
-      </c>
-      <c r="I10">
-        <v>18.100000000000001</v>
-      </c>
-      <c r="J10">
-        <v>21.7</v>
       </c>
       <c r="K10">
         <v>37898681350194</v>
@@ -1546,19 +1546,19 @@
         <v>60</v>
       </c>
       <c r="F11">
+        <v>980</v>
+      </c>
+      <c r="G11">
+        <v>23.5</v>
+      </c>
+      <c r="H11">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="I11">
+        <v>13.5</v>
+      </c>
+      <c r="J11">
         <v>36</v>
-      </c>
-      <c r="G11">
-        <v>980</v>
-      </c>
-      <c r="H11">
-        <v>23.5</v>
-      </c>
-      <c r="I11">
-        <v>16.100000000000001</v>
-      </c>
-      <c r="J11">
-        <v>13.5</v>
       </c>
       <c r="K11">
         <v>17898681350237</v>
@@ -1616,20 +1616,20 @@
       <c r="E12">
         <v>60</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12">
+        <v>980</v>
+      </c>
+      <c r="G12">
+        <v>23.5</v>
+      </c>
+      <c r="H12">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="I12">
+        <v>13.5</v>
+      </c>
+      <c r="J12" t="s">
         <v>123</v>
-      </c>
-      <c r="G12">
-        <v>980</v>
-      </c>
-      <c r="H12">
-        <v>23.5</v>
-      </c>
-      <c r="I12">
-        <v>16.100000000000001</v>
-      </c>
-      <c r="J12">
-        <v>13.5</v>
       </c>
       <c r="K12">
         <v>17898681350237</v>
@@ -1688,19 +1688,19 @@
         <v>24</v>
       </c>
       <c r="F13">
+        <v>1380</v>
+      </c>
+      <c r="G13">
         <v>36</v>
       </c>
-      <c r="G13">
-        <v>1380</v>
-      </c>
       <c r="H13">
+        <v>25</v>
+      </c>
+      <c r="I13">
+        <v>26</v>
+      </c>
+      <c r="J13">
         <v>36</v>
-      </c>
-      <c r="I13">
-        <v>25</v>
-      </c>
-      <c r="J13">
-        <v>26</v>
       </c>
       <c r="K13">
         <v>17898681350244</v>
@@ -1758,20 +1758,20 @@
       <c r="E14">
         <v>24</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14">
+        <v>1380</v>
+      </c>
+      <c r="G14">
+        <v>36</v>
+      </c>
+      <c r="H14">
+        <v>25</v>
+      </c>
+      <c r="I14">
+        <v>26</v>
+      </c>
+      <c r="J14" t="s">
         <v>123</v>
-      </c>
-      <c r="G14">
-        <v>1380</v>
-      </c>
-      <c r="H14">
-        <v>36</v>
-      </c>
-      <c r="I14">
-        <v>25</v>
-      </c>
-      <c r="J14">
-        <v>26</v>
       </c>
       <c r="K14">
         <v>17898681350244</v>
@@ -1829,20 +1829,20 @@
       <c r="E15">
         <v>12</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15">
+        <v>1000</v>
+      </c>
+      <c r="G15">
+        <v>25.1</v>
+      </c>
+      <c r="H15">
+        <v>23.6</v>
+      </c>
+      <c r="I15">
+        <v>13.6</v>
+      </c>
+      <c r="J15" t="s">
         <v>123</v>
-      </c>
-      <c r="G15">
-        <v>1000</v>
-      </c>
-      <c r="H15">
-        <v>25.1</v>
-      </c>
-      <c r="I15">
-        <v>23.6</v>
-      </c>
-      <c r="J15">
-        <v>13.6</v>
       </c>
       <c r="K15">
         <v>17898681350251</v>
@@ -1909,20 +1909,20 @@
       <c r="E16">
         <v>12</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16">
+        <v>1000</v>
+      </c>
+      <c r="G16">
+        <v>25.1</v>
+      </c>
+      <c r="H16">
+        <v>23.6</v>
+      </c>
+      <c r="I16">
+        <v>13.6</v>
+      </c>
+      <c r="J16" t="s">
         <v>123</v>
-      </c>
-      <c r="G16">
-        <v>1000</v>
-      </c>
-      <c r="H16">
-        <v>25.1</v>
-      </c>
-      <c r="I16">
-        <v>23.6</v>
-      </c>
-      <c r="J16">
-        <v>13.6</v>
       </c>
       <c r="K16">
         <v>17898681350251</v>
@@ -1989,20 +1989,20 @@
       <c r="E17">
         <v>12</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17">
+        <v>1000</v>
+      </c>
+      <c r="G17">
+        <v>24.7</v>
+      </c>
+      <c r="H17">
+        <v>24.4</v>
+      </c>
+      <c r="I17">
+        <v>13.7</v>
+      </c>
+      <c r="J17" t="s">
         <v>123</v>
-      </c>
-      <c r="G17">
-        <v>1000</v>
-      </c>
-      <c r="H17">
-        <v>24.7</v>
-      </c>
-      <c r="I17">
-        <v>24.4</v>
-      </c>
-      <c r="J17">
-        <v>13.7</v>
       </c>
       <c r="K17">
         <v>17898681350268</v>
@@ -2070,19 +2070,19 @@
         <v>8</v>
       </c>
       <c r="F18">
-        <v>36</v>
+        <v>790</v>
       </c>
       <c r="G18">
-        <v>790</v>
+        <v>22</v>
       </c>
       <c r="H18">
         <v>22</v>
       </c>
       <c r="I18">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="J18">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="K18">
         <v>17898681350282</v>
@@ -2140,20 +2140,20 @@
       <c r="E19">
         <v>12</v>
       </c>
-      <c r="F19" t="s">
-        <v>123</v>
+      <c r="F19">
+        <v>0.79</v>
       </c>
       <c r="G19">
-        <v>0.79</v>
+        <v>0.22</v>
       </c>
       <c r="H19">
         <v>0.22</v>
       </c>
       <c r="I19">
-        <v>0.22</v>
-      </c>
-      <c r="J19">
         <v>0.08</v>
+      </c>
+      <c r="J19" t="s">
+        <v>123</v>
       </c>
       <c r="K19">
         <v>17898681351654</v>
@@ -2212,19 +2212,19 @@
         <v>72</v>
       </c>
       <c r="F20">
+        <v>1440</v>
+      </c>
+      <c r="G20">
+        <v>42</v>
+      </c>
+      <c r="H20">
+        <v>14.7</v>
+      </c>
+      <c r="I20">
+        <v>14.6</v>
+      </c>
+      <c r="J20">
         <v>36</v>
-      </c>
-      <c r="G20">
-        <v>1440</v>
-      </c>
-      <c r="H20">
-        <v>42</v>
-      </c>
-      <c r="I20">
-        <v>14.7</v>
-      </c>
-      <c r="J20">
-        <v>14.6</v>
       </c>
       <c r="K20">
         <v>17898681350312</v>
@@ -2283,19 +2283,19 @@
         <v>72</v>
       </c>
       <c r="F21">
+        <v>1440</v>
+      </c>
+      <c r="G21">
+        <v>42</v>
+      </c>
+      <c r="H21">
+        <v>14.7</v>
+      </c>
+      <c r="I21">
+        <v>14.6</v>
+      </c>
+      <c r="J21">
         <v>36</v>
-      </c>
-      <c r="G21">
-        <v>1440</v>
-      </c>
-      <c r="H21">
-        <v>42</v>
-      </c>
-      <c r="I21">
-        <v>14.7</v>
-      </c>
-      <c r="J21">
-        <v>14.6</v>
       </c>
       <c r="K21">
         <v>17898681350312</v>
@@ -2354,19 +2354,19 @@
         <v>24</v>
       </c>
       <c r="F22">
+        <v>1740</v>
+      </c>
+      <c r="G22">
+        <v>31.5</v>
+      </c>
+      <c r="H22">
+        <v>16.5</v>
+      </c>
+      <c r="I22">
+        <v>23.5</v>
+      </c>
+      <c r="J22">
         <v>36</v>
-      </c>
-      <c r="G22">
-        <v>1740</v>
-      </c>
-      <c r="H22">
-        <v>31.5</v>
-      </c>
-      <c r="I22">
-        <v>16.5</v>
-      </c>
-      <c r="J22">
-        <v>23.5</v>
       </c>
       <c r="K22">
         <v>17898681350329</v>
@@ -2424,20 +2424,20 @@
       <c r="E23">
         <v>24</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23">
+        <v>1740</v>
+      </c>
+      <c r="G23">
+        <v>31.5</v>
+      </c>
+      <c r="H23">
+        <v>16.5</v>
+      </c>
+      <c r="I23">
+        <v>23.5</v>
+      </c>
+      <c r="J23" t="s">
         <v>123</v>
-      </c>
-      <c r="G23">
-        <v>1740</v>
-      </c>
-      <c r="H23">
-        <v>31.5</v>
-      </c>
-      <c r="I23">
-        <v>16.5</v>
-      </c>
-      <c r="J23">
-        <v>23.5</v>
       </c>
       <c r="K23">
         <v>17898681350329</v>
@@ -2493,19 +2493,19 @@
         <v>60</v>
       </c>
       <c r="F24">
+        <v>1600</v>
+      </c>
+      <c r="G24">
+        <v>16.3</v>
+      </c>
+      <c r="H24">
+        <v>15.7</v>
+      </c>
+      <c r="I24">
+        <v>24.7</v>
+      </c>
+      <c r="J24">
         <v>36</v>
-      </c>
-      <c r="G24">
-        <v>1600</v>
-      </c>
-      <c r="H24">
-        <v>16.3</v>
-      </c>
-      <c r="I24">
-        <v>15.7</v>
-      </c>
-      <c r="J24">
-        <v>24.7</v>
       </c>
       <c r="K24">
         <v>37898681350330</v>
@@ -2564,19 +2564,19 @@
         <v>36</v>
       </c>
       <c r="F25">
+        <v>1670</v>
+      </c>
+      <c r="G25">
+        <v>38.6</v>
+      </c>
+      <c r="H25">
+        <v>20.2</v>
+      </c>
+      <c r="I25">
+        <v>19</v>
+      </c>
+      <c r="J25">
         <v>36</v>
-      </c>
-      <c r="G25">
-        <v>1670</v>
-      </c>
-      <c r="H25">
-        <v>38.6</v>
-      </c>
-      <c r="I25">
-        <v>20.2</v>
-      </c>
-      <c r="J25">
-        <v>19</v>
       </c>
       <c r="K25">
         <v>17898681350619</v>
@@ -2635,19 +2635,19 @@
         <v>24</v>
       </c>
       <c r="F26">
+        <v>1890</v>
+      </c>
+      <c r="G26">
+        <v>32.5</v>
+      </c>
+      <c r="H26">
+        <v>20</v>
+      </c>
+      <c r="I26">
+        <v>25.1</v>
+      </c>
+      <c r="J26">
         <v>36</v>
-      </c>
-      <c r="G26">
-        <v>1890</v>
-      </c>
-      <c r="H26">
-        <v>32.5</v>
-      </c>
-      <c r="I26">
-        <v>20</v>
-      </c>
-      <c r="J26">
-        <v>25.1</v>
       </c>
       <c r="K26">
         <v>17898681350664</v>
@@ -2705,20 +2705,20 @@
       <c r="E27">
         <v>24</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27">
+        <v>1890</v>
+      </c>
+      <c r="G27">
+        <v>32.5</v>
+      </c>
+      <c r="H27">
+        <v>20</v>
+      </c>
+      <c r="I27">
+        <v>25.1</v>
+      </c>
+      <c r="J27" t="s">
         <v>123</v>
-      </c>
-      <c r="G27">
-        <v>1890</v>
-      </c>
-      <c r="H27">
-        <v>32.5</v>
-      </c>
-      <c r="I27">
-        <v>20</v>
-      </c>
-      <c r="J27">
-        <v>25.1</v>
       </c>
       <c r="K27">
         <v>17898681350664</v>
@@ -2777,19 +2777,19 @@
         <v>36</v>
       </c>
       <c r="F28">
+        <v>1890</v>
+      </c>
+      <c r="G28">
+        <v>38.6</v>
+      </c>
+      <c r="H28">
+        <v>20.2</v>
+      </c>
+      <c r="I28">
+        <v>19</v>
+      </c>
+      <c r="J28">
         <v>36</v>
-      </c>
-      <c r="G28">
-        <v>1890</v>
-      </c>
-      <c r="H28">
-        <v>38.6</v>
-      </c>
-      <c r="I28">
-        <v>20.2</v>
-      </c>
-      <c r="J28">
-        <v>19</v>
       </c>
       <c r="K28">
         <v>17898681350718</v>
@@ -2847,20 +2847,20 @@
       <c r="E29">
         <v>36</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29">
+        <v>1890</v>
+      </c>
+      <c r="G29">
+        <v>38.6</v>
+      </c>
+      <c r="H29">
+        <v>20.2</v>
+      </c>
+      <c r="I29">
+        <v>19</v>
+      </c>
+      <c r="J29" t="s">
         <v>123</v>
-      </c>
-      <c r="G29">
-        <v>1890</v>
-      </c>
-      <c r="H29">
-        <v>38.6</v>
-      </c>
-      <c r="I29">
-        <v>20.2</v>
-      </c>
-      <c r="J29">
-        <v>19</v>
       </c>
       <c r="K29">
         <v>17898681350718</v>
@@ -2919,19 +2919,19 @@
         <v>24</v>
       </c>
       <c r="F30">
+        <v>3380</v>
+      </c>
+      <c r="G30">
+        <v>26.1</v>
+      </c>
+      <c r="H30">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="I30">
+        <v>18.3</v>
+      </c>
+      <c r="J30">
         <v>36</v>
-      </c>
-      <c r="G30">
-        <v>3380</v>
-      </c>
-      <c r="H30">
-        <v>26.1</v>
-      </c>
-      <c r="I30">
-        <v>19.399999999999999</v>
-      </c>
-      <c r="J30">
-        <v>18.3</v>
       </c>
       <c r="K30">
         <v>17898681350749</v>
@@ -2990,19 +2990,19 @@
         <v>24</v>
       </c>
       <c r="F31">
+        <v>3.35</v>
+      </c>
+      <c r="G31">
+        <v>0.26</v>
+      </c>
+      <c r="H31">
+        <v>0.2</v>
+      </c>
+      <c r="I31">
+        <v>0.18</v>
+      </c>
+      <c r="J31">
         <v>36</v>
-      </c>
-      <c r="G31">
-        <v>3.35</v>
-      </c>
-      <c r="H31">
-        <v>0.26</v>
-      </c>
-      <c r="I31">
-        <v>0.2</v>
-      </c>
-      <c r="J31">
-        <v>0.18</v>
       </c>
       <c r="K31">
         <v>17898681351609</v>
@@ -3061,19 +3061,19 @@
         <v>32</v>
       </c>
       <c r="F32">
+        <v>3320</v>
+      </c>
+      <c r="G32">
+        <v>33.5</v>
+      </c>
+      <c r="H32">
+        <v>18.7</v>
+      </c>
+      <c r="I32">
+        <v>17</v>
+      </c>
+      <c r="J32">
         <v>36</v>
-      </c>
-      <c r="G32">
-        <v>3320</v>
-      </c>
-      <c r="H32">
-        <v>33.5</v>
-      </c>
-      <c r="I32">
-        <v>18.7</v>
-      </c>
-      <c r="J32">
-        <v>17</v>
       </c>
       <c r="K32">
         <v>17898681350879</v>
@@ -3132,19 +3132,19 @@
         <v>32</v>
       </c>
       <c r="F33">
+        <v>3320</v>
+      </c>
+      <c r="G33">
+        <v>33.5</v>
+      </c>
+      <c r="H33">
+        <v>18.7</v>
+      </c>
+      <c r="I33">
+        <v>17</v>
+      </c>
+      <c r="J33">
         <v>36</v>
-      </c>
-      <c r="G33">
-        <v>3320</v>
-      </c>
-      <c r="H33">
-        <v>33.5</v>
-      </c>
-      <c r="I33">
-        <v>18.7</v>
-      </c>
-      <c r="J33">
-        <v>17</v>
       </c>
       <c r="K33">
         <v>17898681350879</v>
@@ -3202,20 +3202,20 @@
       <c r="E34">
         <v>18</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34">
+        <v>590</v>
+      </c>
+      <c r="G34">
+        <v>18</v>
+      </c>
+      <c r="H34">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="I34">
+        <v>15.1</v>
+      </c>
+      <c r="J34" t="s">
         <v>123</v>
-      </c>
-      <c r="G34">
-        <v>590</v>
-      </c>
-      <c r="H34">
-        <v>18</v>
-      </c>
-      <c r="I34">
-        <v>16.600000000000001</v>
-      </c>
-      <c r="J34">
-        <v>15.1</v>
       </c>
       <c r="K34">
         <v>17898681350923</v>
@@ -3282,20 +3282,20 @@
       <c r="E35">
         <v>18</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35">
+        <v>590</v>
+      </c>
+      <c r="G35">
+        <v>18</v>
+      </c>
+      <c r="H35">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="I35">
+        <v>15.1</v>
+      </c>
+      <c r="J35" t="s">
         <v>123</v>
-      </c>
-      <c r="G35">
-        <v>590</v>
-      </c>
-      <c r="H35">
-        <v>18</v>
-      </c>
-      <c r="I35">
-        <v>16.600000000000001</v>
-      </c>
-      <c r="J35">
-        <v>15.1</v>
       </c>
       <c r="K35">
         <v>17898681350923</v>
@@ -3363,19 +3363,19 @@
         <v>96</v>
       </c>
       <c r="F36">
+        <v>3700</v>
+      </c>
+      <c r="G36">
+        <v>22.6</v>
+      </c>
+      <c r="H36">
+        <v>17.3</v>
+      </c>
+      <c r="I36">
+        <v>23.1</v>
+      </c>
+      <c r="J36">
         <v>36</v>
-      </c>
-      <c r="G36">
-        <v>3700</v>
-      </c>
-      <c r="H36">
-        <v>22.6</v>
-      </c>
-      <c r="I36">
-        <v>17.3</v>
-      </c>
-      <c r="J36">
-        <v>23.1</v>
       </c>
       <c r="K36">
         <v>17898681350930</v>
@@ -3433,20 +3433,20 @@
       <c r="E37">
         <v>96</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37">
+        <v>3700</v>
+      </c>
+      <c r="G37">
+        <v>22.6</v>
+      </c>
+      <c r="H37">
+        <v>17.3</v>
+      </c>
+      <c r="I37">
+        <v>23.1</v>
+      </c>
+      <c r="J37" t="s">
         <v>123</v>
-      </c>
-      <c r="G37">
-        <v>3700</v>
-      </c>
-      <c r="H37">
-        <v>22.6</v>
-      </c>
-      <c r="I37">
-        <v>17.3</v>
-      </c>
-      <c r="J37">
-        <v>23.1</v>
       </c>
       <c r="K37">
         <v>17898681350930</v>
@@ -3505,19 +3505,19 @@
         <v>96</v>
       </c>
       <c r="F38">
+        <v>2420</v>
+      </c>
+      <c r="G38">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="H38">
+        <v>19.8</v>
+      </c>
+      <c r="I38">
+        <v>13.4</v>
+      </c>
+      <c r="J38">
         <v>36</v>
-      </c>
-      <c r="G38">
-        <v>2420</v>
-      </c>
-      <c r="H38">
-        <v>38.299999999999997</v>
-      </c>
-      <c r="I38">
-        <v>19.8</v>
-      </c>
-      <c r="J38">
-        <v>13.4</v>
       </c>
       <c r="K38">
         <v>17898681351036</v>
@@ -3575,20 +3575,20 @@
       <c r="E39">
         <v>96</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39">
+        <v>2420</v>
+      </c>
+      <c r="G39">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="H39">
+        <v>19.8</v>
+      </c>
+      <c r="I39">
+        <v>13.4</v>
+      </c>
+      <c r="J39" t="s">
         <v>123</v>
-      </c>
-      <c r="G39">
-        <v>2420</v>
-      </c>
-      <c r="H39">
-        <v>38.299999999999997</v>
-      </c>
-      <c r="I39">
-        <v>19.8</v>
-      </c>
-      <c r="J39">
-        <v>13.4</v>
       </c>
       <c r="K39">
         <v>17898681351036</v>
@@ -3647,19 +3647,19 @@
         <v>24</v>
       </c>
       <c r="F40">
+        <v>2710</v>
+      </c>
+      <c r="G40">
+        <v>26</v>
+      </c>
+      <c r="H40">
+        <v>19.7</v>
+      </c>
+      <c r="I40">
+        <v>17.5</v>
+      </c>
+      <c r="J40">
         <v>36</v>
-      </c>
-      <c r="G40">
-        <v>2710</v>
-      </c>
-      <c r="H40">
-        <v>26</v>
-      </c>
-      <c r="I40">
-        <v>19.7</v>
-      </c>
-      <c r="J40">
-        <v>17.5</v>
       </c>
       <c r="K40">
         <v>17898681351173</v>
@@ -3718,19 +3718,19 @@
         <v>12</v>
       </c>
       <c r="F41">
+        <v>2000</v>
+      </c>
+      <c r="G41">
+        <v>22.7</v>
+      </c>
+      <c r="H41">
+        <v>24.4</v>
+      </c>
+      <c r="I41">
+        <v>11.4</v>
+      </c>
+      <c r="J41">
         <v>36</v>
-      </c>
-      <c r="G41">
-        <v>2000</v>
-      </c>
-      <c r="H41">
-        <v>22.7</v>
-      </c>
-      <c r="I41">
-        <v>24.4</v>
-      </c>
-      <c r="J41">
-        <v>11.4</v>
       </c>
       <c r="K41">
         <v>17898681351180</v>
@@ -3788,20 +3788,20 @@
       <c r="E42">
         <v>12</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42">
+        <v>2000</v>
+      </c>
+      <c r="G42">
+        <v>22.7</v>
+      </c>
+      <c r="H42">
+        <v>24.4</v>
+      </c>
+      <c r="I42">
+        <v>11.4</v>
+      </c>
+      <c r="J42" t="s">
         <v>123</v>
-      </c>
-      <c r="G42">
-        <v>2000</v>
-      </c>
-      <c r="H42">
-        <v>22.7</v>
-      </c>
-      <c r="I42">
-        <v>24.4</v>
-      </c>
-      <c r="J42">
-        <v>11.4</v>
       </c>
       <c r="K42">
         <v>17898681351180</v>
@@ -3860,19 +3860,19 @@
         <v>12</v>
       </c>
       <c r="F43">
+        <v>1520</v>
+      </c>
+      <c r="G43">
+        <v>23</v>
+      </c>
+      <c r="H43">
+        <v>22.7</v>
+      </c>
+      <c r="I43">
+        <v>11.4</v>
+      </c>
+      <c r="J43">
         <v>36</v>
-      </c>
-      <c r="G43">
-        <v>1520</v>
-      </c>
-      <c r="H43">
-        <v>23</v>
-      </c>
-      <c r="I43">
-        <v>22.7</v>
-      </c>
-      <c r="J43">
-        <v>11.4</v>
       </c>
       <c r="K43">
         <v>17898681351197</v>
@@ -3931,19 +3931,19 @@
         <v>20</v>
       </c>
       <c r="F44">
+        <v>1460</v>
+      </c>
+      <c r="G44">
+        <v>21.4</v>
+      </c>
+      <c r="H44">
+        <v>15.1</v>
+      </c>
+      <c r="I44">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="J44">
         <v>36</v>
-      </c>
-      <c r="G44">
-        <v>1460</v>
-      </c>
-      <c r="H44">
-        <v>21.4</v>
-      </c>
-      <c r="I44">
-        <v>15.1</v>
-      </c>
-      <c r="J44">
-        <v>32.200000000000003</v>
       </c>
       <c r="K44">
         <v>17898681351302</v>
@@ -4001,20 +4001,20 @@
       <c r="E45">
         <v>20</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45">
+        <v>1460</v>
+      </c>
+      <c r="G45">
+        <v>21.4</v>
+      </c>
+      <c r="H45">
+        <v>15.1</v>
+      </c>
+      <c r="I45">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="J45" t="s">
         <v>123</v>
-      </c>
-      <c r="G45">
-        <v>1460</v>
-      </c>
-      <c r="H45">
-        <v>21.4</v>
-      </c>
-      <c r="I45">
-        <v>15.1</v>
-      </c>
-      <c r="J45">
-        <v>32.200000000000003</v>
       </c>
       <c r="K45">
         <v>17898681351302</v>
@@ -4073,19 +4073,19 @@
         <v>24</v>
       </c>
       <c r="F46">
+        <v>3300</v>
+      </c>
+      <c r="G46">
+        <v>26.5</v>
+      </c>
+      <c r="H46">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="I46">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="J46">
         <v>36</v>
-      </c>
-      <c r="G46">
-        <v>3300</v>
-      </c>
-      <c r="H46">
-        <v>26.5</v>
-      </c>
-      <c r="I46">
-        <v>20.100000000000001</v>
-      </c>
-      <c r="J46">
-        <v>17.399999999999999</v>
       </c>
       <c r="K46">
         <v>17898681351364</v>
@@ -4144,19 +4144,19 @@
         <v>24</v>
       </c>
       <c r="F47">
+        <v>3394</v>
+      </c>
+      <c r="G47">
+        <v>25.6</v>
+      </c>
+      <c r="H47">
+        <v>19.7</v>
+      </c>
+      <c r="I47">
+        <v>17.5</v>
+      </c>
+      <c r="J47">
         <v>36</v>
-      </c>
-      <c r="G47">
-        <v>3394</v>
-      </c>
-      <c r="H47">
-        <v>25.6</v>
-      </c>
-      <c r="I47">
-        <v>19.7</v>
-      </c>
-      <c r="J47">
-        <v>17.5</v>
       </c>
       <c r="K47">
         <v>17898681351371</v>
@@ -4214,20 +4214,20 @@
       <c r="E48">
         <v>24</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48">
+        <v>3394</v>
+      </c>
+      <c r="G48">
+        <v>25.6</v>
+      </c>
+      <c r="H48">
+        <v>19.7</v>
+      </c>
+      <c r="I48">
+        <v>17.5</v>
+      </c>
+      <c r="J48" t="s">
         <v>123</v>
-      </c>
-      <c r="G48">
-        <v>3394</v>
-      </c>
-      <c r="H48">
-        <v>25.6</v>
-      </c>
-      <c r="I48">
-        <v>19.7</v>
-      </c>
-      <c r="J48">
-        <v>17.5</v>
       </c>
       <c r="K48">
         <v>17898681351371</v>
@@ -4286,19 +4286,19 @@
         <v>4</v>
       </c>
       <c r="F49">
-        <v>36</v>
+        <v>1840</v>
       </c>
       <c r="G49">
-        <v>1840</v>
+        <v>20.3</v>
       </c>
       <c r="H49">
         <v>20.3</v>
       </c>
       <c r="I49">
-        <v>20.3</v>
+        <v>0.11</v>
       </c>
       <c r="J49">
-        <v>0.11</v>
+        <v>36</v>
       </c>
       <c r="Q49">
         <v>7898681351428</v>
@@ -4339,19 +4339,19 @@
         <v>27</v>
       </c>
       <c r="F50">
+        <v>2420</v>
+      </c>
+      <c r="G50">
+        <v>51.2</v>
+      </c>
+      <c r="H50">
+        <v>25.1</v>
+      </c>
+      <c r="I50">
+        <v>18.5</v>
+      </c>
+      <c r="J50">
         <v>36</v>
-      </c>
-      <c r="G50">
-        <v>2420</v>
-      </c>
-      <c r="H50">
-        <v>51.2</v>
-      </c>
-      <c r="I50">
-        <v>25.1</v>
-      </c>
-      <c r="J50">
-        <v>18.5</v>
       </c>
       <c r="K50">
         <v>37898681351467</v>
@@ -4409,20 +4409,20 @@
       <c r="E51">
         <v>27</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F51">
+        <v>2420</v>
+      </c>
+      <c r="G51">
+        <v>51.2</v>
+      </c>
+      <c r="H51">
+        <v>25.1</v>
+      </c>
+      <c r="I51">
+        <v>18.5</v>
+      </c>
+      <c r="J51" t="s">
         <v>123</v>
-      </c>
-      <c r="G51">
-        <v>2420</v>
-      </c>
-      <c r="H51">
-        <v>51.2</v>
-      </c>
-      <c r="I51">
-        <v>25.1</v>
-      </c>
-      <c r="J51">
-        <v>18.5</v>
       </c>
       <c r="K51">
         <v>37898681351467</v>
@@ -4481,19 +4481,19 @@
         <v>24</v>
       </c>
       <c r="F52">
+        <v>1400</v>
+      </c>
+      <c r="G52">
+        <v>37.299999999999997</v>
+      </c>
+      <c r="H52">
+        <v>25</v>
+      </c>
+      <c r="I52">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="J52">
         <v>36</v>
-      </c>
-      <c r="G52">
-        <v>1400</v>
-      </c>
-      <c r="H52">
-        <v>37.299999999999997</v>
-      </c>
-      <c r="I52">
-        <v>25</v>
-      </c>
-      <c r="J52">
-        <v>16.100000000000001</v>
       </c>
       <c r="K52">
         <v>17898681351470</v>
@@ -4551,20 +4551,20 @@
       <c r="E53">
         <v>24</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F53">
+        <v>1400</v>
+      </c>
+      <c r="G53">
+        <v>37.299999999999997</v>
+      </c>
+      <c r="H53">
+        <v>25</v>
+      </c>
+      <c r="I53">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="J53" t="s">
         <v>123</v>
-      </c>
-      <c r="G53">
-        <v>1400</v>
-      </c>
-      <c r="H53">
-        <v>37.299999999999997</v>
-      </c>
-      <c r="I53">
-        <v>25</v>
-      </c>
-      <c r="J53">
-        <v>16.100000000000001</v>
       </c>
       <c r="K53">
         <v>17898681351470</v>
@@ -4623,19 +4623,19 @@
         <v>40</v>
       </c>
       <c r="F54">
+        <v>1990</v>
+      </c>
+      <c r="G54">
+        <v>14</v>
+      </c>
+      <c r="H54">
+        <v>21</v>
+      </c>
+      <c r="I54">
+        <v>17</v>
+      </c>
+      <c r="J54">
         <v>24</v>
-      </c>
-      <c r="G54">
-        <v>1990</v>
-      </c>
-      <c r="H54">
-        <v>14</v>
-      </c>
-      <c r="I54">
-        <v>21</v>
-      </c>
-      <c r="J54">
-        <v>17</v>
       </c>
       <c r="K54">
         <v>17898681351494</v>
@@ -4694,19 +4694,19 @@
         <v>24</v>
       </c>
       <c r="F55">
+        <v>2190</v>
+      </c>
+      <c r="G55">
+        <v>27</v>
+      </c>
+      <c r="H55">
+        <v>21</v>
+      </c>
+      <c r="I55">
+        <v>11</v>
+      </c>
+      <c r="J55">
         <v>36</v>
-      </c>
-      <c r="G55">
-        <v>2190</v>
-      </c>
-      <c r="H55">
-        <v>27</v>
-      </c>
-      <c r="I55">
-        <v>21</v>
-      </c>
-      <c r="J55">
-        <v>11</v>
       </c>
       <c r="K55">
         <v>17898681351500</v>
@@ -4764,20 +4764,20 @@
       <c r="E56">
         <v>24</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F56">
+        <v>2190</v>
+      </c>
+      <c r="G56">
+        <v>27</v>
+      </c>
+      <c r="H56">
+        <v>21</v>
+      </c>
+      <c r="I56">
+        <v>11</v>
+      </c>
+      <c r="J56" t="s">
         <v>123</v>
-      </c>
-      <c r="G56">
-        <v>2190</v>
-      </c>
-      <c r="H56">
-        <v>27</v>
-      </c>
-      <c r="I56">
-        <v>21</v>
-      </c>
-      <c r="J56">
-        <v>11</v>
       </c>
       <c r="K56">
         <v>17898681351500</v>
@@ -4836,19 +4836,19 @@
         <v>120</v>
       </c>
       <c r="F57">
-        <v>24</v>
+        <v>1.2</v>
       </c>
       <c r="G57">
-        <v>1.2</v>
+        <v>0.42</v>
       </c>
       <c r="H57">
-        <v>0.42</v>
+        <v>0.19</v>
       </c>
       <c r="I57">
         <v>0.19</v>
       </c>
       <c r="J57">
-        <v>0.19</v>
+        <v>24</v>
       </c>
       <c r="K57">
         <v>17898681351647</v>
@@ -4916,19 +4916,19 @@
         <v>120</v>
       </c>
       <c r="F58">
-        <v>24</v>
+        <v>1.2</v>
       </c>
       <c r="G58">
-        <v>1.2</v>
+        <v>0.42</v>
       </c>
       <c r="H58">
-        <v>0.42</v>
+        <v>0.19</v>
       </c>
       <c r="I58">
         <v>0.19</v>
       </c>
       <c r="J58">
-        <v>0.19</v>
+        <v>24</v>
       </c>
       <c r="K58">
         <v>17898681351647</v>
@@ -4996,19 +4996,19 @@
         <v>24</v>
       </c>
       <c r="F59">
+        <v>3200</v>
+      </c>
+      <c r="G59">
+        <v>32.4</v>
+      </c>
+      <c r="H59">
+        <v>21.7</v>
+      </c>
+      <c r="I59">
+        <v>14.6</v>
+      </c>
+      <c r="J59">
         <v>36</v>
-      </c>
-      <c r="G59">
-        <v>3200</v>
-      </c>
-      <c r="H59">
-        <v>32.4</v>
-      </c>
-      <c r="I59">
-        <v>21.7</v>
-      </c>
-      <c r="J59">
-        <v>14.6</v>
       </c>
       <c r="K59">
         <v>17898681351531</v>
@@ -5067,19 +5067,19 @@
         <v>60</v>
       </c>
       <c r="F60">
+        <v>1.88</v>
+      </c>
+      <c r="G60">
+        <v>25.3</v>
+      </c>
+      <c r="H60">
+        <v>18.5</v>
+      </c>
+      <c r="I60">
+        <v>22.7</v>
+      </c>
+      <c r="J60">
         <v>36</v>
-      </c>
-      <c r="G60">
-        <v>1.88</v>
-      </c>
-      <c r="H60">
-        <v>25.3</v>
-      </c>
-      <c r="I60">
-        <v>18.5</v>
-      </c>
-      <c r="J60">
-        <v>22.7</v>
       </c>
       <c r="K60">
         <v>17898681351548</v>
@@ -5137,20 +5137,20 @@
       <c r="E61">
         <v>60</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F61">
+        <v>1.88</v>
+      </c>
+      <c r="G61">
+        <v>25.3</v>
+      </c>
+      <c r="H61">
+        <v>18.5</v>
+      </c>
+      <c r="I61">
+        <v>22.7</v>
+      </c>
+      <c r="J61" t="s">
         <v>123</v>
-      </c>
-      <c r="G61">
-        <v>1.88</v>
-      </c>
-      <c r="H61">
-        <v>25.3</v>
-      </c>
-      <c r="I61">
-        <v>18.5</v>
-      </c>
-      <c r="J61">
-        <v>22.7</v>
       </c>
       <c r="K61">
         <v>17898681351548</v>
@@ -5209,19 +5209,19 @@
         <v>72</v>
       </c>
       <c r="F62">
+        <v>5600</v>
+      </c>
+      <c r="G62">
+        <v>31</v>
+      </c>
+      <c r="H62">
+        <v>26.4</v>
+      </c>
+      <c r="I62">
+        <v>23</v>
+      </c>
+      <c r="J62">
         <v>36</v>
-      </c>
-      <c r="G62">
-        <v>5600</v>
-      </c>
-      <c r="H62">
-        <v>31</v>
-      </c>
-      <c r="I62">
-        <v>26.4</v>
-      </c>
-      <c r="J62">
-        <v>23</v>
       </c>
       <c r="K62">
         <v>17898681351555</v>
@@ -5280,19 +5280,19 @@
         <v>72</v>
       </c>
       <c r="F63">
+        <v>1530</v>
+      </c>
+      <c r="G63">
+        <v>41.7</v>
+      </c>
+      <c r="H63">
+        <v>14.6</v>
+      </c>
+      <c r="I63">
+        <v>14.7</v>
+      </c>
+      <c r="J63">
         <v>36</v>
-      </c>
-      <c r="G63">
-        <v>1530</v>
-      </c>
-      <c r="H63">
-        <v>41.7</v>
-      </c>
-      <c r="I63">
-        <v>14.6</v>
-      </c>
-      <c r="J63">
-        <v>14.7</v>
       </c>
       <c r="K63">
         <v>17898681351562</v>
@@ -5357,19 +5357,19 @@
         <v>72</v>
       </c>
       <c r="F64">
+        <v>1530</v>
+      </c>
+      <c r="G64">
+        <v>41.7</v>
+      </c>
+      <c r="H64">
+        <v>14.6</v>
+      </c>
+      <c r="I64">
+        <v>14.7</v>
+      </c>
+      <c r="J64">
         <v>36</v>
-      </c>
-      <c r="G64">
-        <v>1530</v>
-      </c>
-      <c r="H64">
-        <v>41.7</v>
-      </c>
-      <c r="I64">
-        <v>14.6</v>
-      </c>
-      <c r="J64">
-        <v>14.7</v>
       </c>
       <c r="K64">
         <v>17898681351562</v>
@@ -5433,20 +5433,20 @@
       <c r="E65">
         <v>90</v>
       </c>
-      <c r="F65" t="s">
-        <v>123</v>
+      <c r="F65">
+        <v>2160</v>
       </c>
       <c r="G65">
-        <v>2160</v>
+        <v>45</v>
       </c>
       <c r="H65">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="I65">
         <v>16</v>
       </c>
-      <c r="J65">
-        <v>16</v>
+      <c r="J65" t="s">
+        <v>123</v>
       </c>
       <c r="K65">
         <v>17898681351579</v>
@@ -5514,19 +5514,19 @@
         <v>36</v>
       </c>
       <c r="F66">
+        <v>2180</v>
+      </c>
+      <c r="G66">
         <v>36</v>
       </c>
-      <c r="G66">
-        <v>2180</v>
-      </c>
       <c r="H66">
+        <v>19</v>
+      </c>
+      <c r="I66">
+        <v>38.5</v>
+      </c>
+      <c r="J66">
         <v>36</v>
-      </c>
-      <c r="I66">
-        <v>19</v>
-      </c>
-      <c r="J66">
-        <v>38.5</v>
       </c>
       <c r="K66">
         <v>17898681351760</v>
@@ -5585,19 +5585,19 @@
         <v>60</v>
       </c>
       <c r="F67">
+        <v>1112</v>
+      </c>
+      <c r="G67">
+        <v>25.5</v>
+      </c>
+      <c r="H67">
+        <v>13.5</v>
+      </c>
+      <c r="I67">
+        <v>18</v>
+      </c>
+      <c r="J67">
         <v>24</v>
-      </c>
-      <c r="G67">
-        <v>1112</v>
-      </c>
-      <c r="H67">
-        <v>25.5</v>
-      </c>
-      <c r="I67">
-        <v>13.5</v>
-      </c>
-      <c r="J67">
-        <v>18</v>
       </c>
       <c r="K67">
         <v>17898681351630</v>
@@ -5656,19 +5656,19 @@
         <v>24</v>
       </c>
       <c r="F68">
+        <v>1330</v>
+      </c>
+      <c r="G68">
+        <v>35.5</v>
+      </c>
+      <c r="H68">
+        <v>16.5</v>
+      </c>
+      <c r="I68">
+        <v>23.5</v>
+      </c>
+      <c r="J68">
         <v>24</v>
-      </c>
-      <c r="G68">
-        <v>1330</v>
-      </c>
-      <c r="H68">
-        <v>35.5</v>
-      </c>
-      <c r="I68">
-        <v>16.5</v>
-      </c>
-      <c r="J68">
-        <v>23.5</v>
       </c>
       <c r="K68">
         <v>17898681351708</v>

</xml_diff>